<commit_message>
Add Finviz breadth percentages
</commit_message>
<xml_diff>
--- a/finviz_breadth.xlsx
+++ b/finviz_breadth.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -425,6 +425,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,17 +444,37 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>New High %</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>New Low</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>New Low %</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Advancing</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Advancing %</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Declining</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Declining %</t>
         </is>
       </c>
     </row>
@@ -467,17 +491,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>50.6%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>256</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>49.4%</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>2368</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>42.3%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>3015</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>53.9%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Finviz breadth data
</commit_message>
<xml_diff>
--- a/finviz_breadth.xlsx
+++ b/finviz_breadth.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,53 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>50.6%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>49.4%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2368</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>42.3%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>3015</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>53.9%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>